<commit_message>
add: save_products validation test + initial parametrize
</commit_message>
<xml_diff>
--- a/docs/CasosTeste.xlsx
+++ b/docs/CasosTeste.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\Repo\product-management-app\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E6FD937-C587-4E53-BF71-4FD207544977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684A9BEE-E6C7-406F-8516-0D03BF3BE898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="0" windowWidth="10455" windowHeight="10800" xr2:uid="{1C90CB3A-62C0-4AFC-9C95-1D254DB19A7C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{1C90CB3A-62C0-4AFC-9C95-1D254DB19A7C}"/>
   </bookViews>
   <sheets>
     <sheet name="CadastrarProduto" sheetId="1" r:id="rId1"/>
     <sheet name="Planilha2" sheetId="2" r:id="rId2"/>
-    <sheet name="EditarProduto" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,15 +26,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="234">
   <si>
     <t>Casos de Teste</t>
   </si>
   <si>
     <t>ID</t>
-  </si>
-  <si>
-    <t>Requisito</t>
   </si>
   <si>
     <t>Cenário</t>
@@ -825,6 +821,18 @@
   </si>
   <si>
     <t>Cadastrar um nome de produto com 20 caracteres</t>
+  </si>
+  <si>
+    <t>Nível de Teste</t>
+  </si>
+  <si>
+    <t>Funcional</t>
+  </si>
+  <si>
+    <t>RF</t>
+  </si>
+  <si>
+    <t>Unidade</t>
   </si>
 </sst>
 </file>
@@ -972,26 +980,36 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Título 2" xfId="1" builtinId="17"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="19">
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
       <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.39994506668294322"/>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thick">
+          <color theme="0"/>
+        </left>
+        <right style="thick">
+          <color theme="0"/>
+        </right>
+        <top style="thick">
+          <color theme="0"/>
+        </top>
+        <bottom style="thick">
+          <color theme="0"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1268,256 +1286,6 @@
     <dxf>
       <border outline="0">
         <top style="thick">
-          <color rgb="FFFFFFFF"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thick">
-          <color rgb="FFA2B8E1"/>
-        </top>
-        <bottom style="thick">
-          <color rgb="FFFFFFFF"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FFDBDBDB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thick">
-          <color rgb="FFA2B8E1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thick">
-          <color theme="0"/>
-        </left>
-        <right style="thick">
-          <color theme="0"/>
-        </right>
-        <top style="thick">
-          <color theme="0"/>
-        </top>
-        <bottom style="thick">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thick">
-          <color theme="0"/>
-        </left>
-        <right style="thick">
-          <color theme="0"/>
-        </right>
-        <top style="thick">
-          <color theme="0"/>
-        </top>
-        <bottom style="thick">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thick">
-          <color theme="0"/>
-        </left>
-        <right style="thick">
-          <color theme="0"/>
-        </right>
-        <top style="thick">
-          <color theme="0"/>
-        </top>
-        <bottom style="thick">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thick">
-          <color theme="0"/>
-        </left>
-        <right style="thick">
-          <color theme="0"/>
-        </right>
-        <top style="thick">
-          <color theme="0"/>
-        </top>
-        <bottom style="thick">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thick">
-          <color theme="0"/>
-        </left>
-        <right style="thick">
-          <color theme="0"/>
-        </right>
-        <top style="thick">
-          <color theme="0"/>
-        </top>
-        <bottom style="thick">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thick">
-          <color theme="0"/>
-        </left>
-        <right style="thick">
-          <color theme="0"/>
-        </right>
-        <top style="thick">
-          <color theme="0"/>
-        </top>
-        <bottom style="thick">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thick">
-          <color theme="0"/>
-        </left>
-        <right style="thick">
-          <color theme="0"/>
-        </right>
-        <top style="thick">
-          <color theme="0"/>
-        </top>
-        <bottom style="thick">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thick">
-          <color theme="0"/>
-        </left>
-        <right style="thick">
-          <color theme="0"/>
-        </right>
-        <top style="thick">
-          <color theme="0"/>
-        </top>
-        <bottom style="thick">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thick">
-          <color theme="0"/>
-        </left>
-        <right style="thick">
-          <color theme="0"/>
-        </right>
-        <top style="thick">
-          <color theme="0"/>
-        </top>
-        <bottom style="thick">
-          <color theme="0"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thick">
           <color theme="0"/>
         </top>
       </border>
@@ -1561,42 +1329,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7529F5F6-7101-425A-86FE-98BCE73E6CC7}" name="Tabela3" displayName="Tabela3" ref="D4:L71" totalsRowShown="0" dataDxfId="30" headerRowBorderDxfId="31" tableBorderDxfId="29" totalsRowBorderDxfId="28" headerRowCellStyle="Título 2">
-  <autoFilter ref="D4:L71" xr:uid="{7529F5F6-7101-425A-86FE-98BCE73E6CC7}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7529F5F6-7101-425A-86FE-98BCE73E6CC7}" name="Tabela3" displayName="Tabela3" ref="D4:M71" totalsRowShown="0" dataDxfId="17" headerRowBorderDxfId="18" tableBorderDxfId="16" totalsRowBorderDxfId="15" headerRowCellStyle="Título 2">
+  <autoFilter ref="D4:M71" xr:uid="{7529F5F6-7101-425A-86FE-98BCE73E6CC7}">
     <filterColumn colId="1">
       <customFilters>
         <customFilter val="*Cadastrar*"/>
       </customFilters>
     </filterColumn>
   </autoFilter>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{A1BDB3C3-3C77-43F5-8EEB-251483113840}" name="ID" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{CC86DED9-FD31-4CFE-8F71-D12B00A8C63C}" name="Cenário" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{89A7CD85-A211-4621-98A5-AC6DC5C8CBD3}" name="Requisito" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{58B3439F-248E-459D-BF23-4F819BF6E6CF}" name="Critério" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{2F6AA3F2-86BC-4B8E-A72C-8875F1F5E6CA}" name="Pré-condição" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{9D74B700-6AE1-453E-93DA-2B74929327DA}" name="Passos" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{85378303-32EA-4A42-B7A6-D80BAFEDB568}" name="Resultados Esperados" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{D4F1EF2C-B773-4C7A-91AB-3B1EE9B79FA8}" name="Status" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{5F57F91E-F603-4252-8D61-5DEACB70EF9A}" name="Resultado Obtido" dataDxfId="19"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6B9974CB-E023-4E72-A0A3-D3EB9C34E083}" name="Tabela36" displayName="Tabela36" ref="C3:K15" totalsRowShown="0" dataDxfId="17" headerRowBorderDxfId="18" tableBorderDxfId="16" totalsRowBorderDxfId="15" headerRowCellStyle="Título 2">
-  <autoFilter ref="C3:K15" xr:uid="{6B9974CB-E023-4E72-A0A3-D3EB9C34E083}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{2E9F1127-6DD3-4DC1-ADEA-D3CBDD2B3A51}" name="ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{C69961BE-6CD0-46EA-9D26-500754BC2D92}" name="Cenário" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{7B8F0275-1692-46B7-882F-A018646778F7}" name="Requisito" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{DB2A4F99-0EC4-41BD-B63D-FBC8206EC00B}" name="Critério" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{E8ABA42B-6F82-414C-98E8-1BF798C27637}" name="Pré-condição" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{E67F0553-914B-4B85-847D-88A1138A7067}" name="Passos" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{8F884CC2-3BD4-4771-8DC3-C3F8579FACCF}" name="Resultados Esperados" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{2854A912-91D0-43B2-8462-C9C9D4BD3568}" name="Status" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{B37A25EA-828F-4E47-A994-E1DAC36FF66A}" name="Resultado Obtido" dataDxfId="6"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{A1BDB3C3-3C77-43F5-8EEB-251483113840}" name="ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{CC86DED9-FD31-4CFE-8F71-D12B00A8C63C}" name="Cenário" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{89A7CD85-A211-4621-98A5-AC6DC5C8CBD3}" name="RF" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{58B3439F-248E-459D-BF23-4F819BF6E6CF}" name="Critério" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{2F6AA3F2-86BC-4B8E-A72C-8875F1F5E6CA}" name="Pré-condição" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{9D74B700-6AE1-453E-93DA-2B74929327DA}" name="Passos" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{85378303-32EA-4A42-B7A6-D80BAFEDB568}" name="Resultados Esperados" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{D4F1EF2C-B773-4C7A-91AB-3B1EE9B79FA8}" name="Status" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{5F57F91E-F603-4252-8D61-5DEACB70EF9A}" name="Resultado Obtido" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{2948477C-3111-49EB-80FC-662CB6D2B52A}" name="Nível de Teste" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1899,22 +1650,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74F0531C-02C9-4914-AA9B-2D861DBE9348}">
-  <dimension ref="C3:L71"/>
+  <dimension ref="C3:M71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.140625" customWidth="1"/>
+    <col min="2" max="2" width="1.42578125" customWidth="1"/>
     <col min="3" max="3" width="2.140625" customWidth="1"/>
-    <col min="5" max="5" width="47.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" customWidth="1"/>
-    <col min="7" max="7" width="11.28515625" customWidth="1"/>
-    <col min="8" max="8" width="68.85546875" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" customWidth="1"/>
+    <col min="5" max="5" width="29.140625" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" customWidth="1"/>
     <col min="9" max="9" width="36.5703125" customWidth="1"/>
-    <col min="10" max="10" width="83.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="34.85546875" customWidth="1"/>
+    <col min="10" max="10" width="19.85546875" customWidth="1"/>
+    <col min="11" max="11" width="10.140625" customWidth="1"/>
+    <col min="12" max="12" width="18.42578125" customWidth="1"/>
+    <col min="13" max="13" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:12" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="3:13" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1927,569 +1681,624 @@
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="3:12" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="3:13" ht="36" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C4" s="3"/>
       <c r="D4" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="K4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="5" spans="3:12" ht="179.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L4" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="M4" s="15" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="5" spans="3:13" ht="162.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C5" s="1"/>
       <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="J5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>13</v>
-      </c>
       <c r="K5" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="6" spans="3:12" ht="151.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+      <c r="M5" s="12" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="6" spans="3:13" ht="214.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C6" s="1"/>
       <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="F6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="H6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="J6" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>19</v>
-      </c>
       <c r="K6" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="7" spans="3:12" ht="169.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+      <c r="M6" s="6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="7" spans="3:13" ht="169.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C7" s="1"/>
       <c r="D7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>21</v>
-      </c>
       <c r="F7" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H7" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="I7" s="6" t="s">
-        <v>102</v>
-      </c>
       <c r="J7" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L7" s="15" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="8" spans="3:12" ht="167.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="8" spans="3:13" ht="167.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C8" s="1"/>
       <c r="D8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="J8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>25</v>
-      </c>
       <c r="K8" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="L8" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="L8" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="9" spans="3:12" ht="150" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M8" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="9" spans="3:13" ht="150" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C9" s="1"/>
       <c r="D9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="J9" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="K9" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="10" spans="3:12" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10" spans="3:13" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C10" s="1"/>
       <c r="D10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="J10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="K10" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="11" spans="3:12" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="11" spans="3:13" ht="181.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C11" s="1"/>
       <c r="D11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="J11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I11" s="6" t="s">
+      <c r="K11" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="L11" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="J11" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L11" s="6" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="12" spans="3:12" ht="62.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M11" s="6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="12" spans="3:13" ht="62.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C12" s="1"/>
       <c r="D12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>33</v>
+      <c r="J12" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L12" s="2"/>
-    </row>
-    <row r="13" spans="3:12" ht="297.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M12" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="13" spans="3:13" ht="297.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C13" s="1"/>
       <c r="D13" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>33</v>
+        <v>124</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L13" s="2"/>
-    </row>
-    <row r="14" spans="3:12" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M13" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="14" spans="3:13" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C14" s="1"/>
       <c r="D14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="6" t="s">
-        <v>41</v>
-      </c>
       <c r="F14" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>17</v>
+        <v>27</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>33</v>
+        <v>107</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="15" spans="3:12" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="15" spans="3:13" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C15" s="1"/>
       <c r="D15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="J15" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I15" s="6" t="s">
+      <c r="K15" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="L15" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="J15" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="16" spans="3:12" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M15" s="6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="16" spans="3:13" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C16" s="1"/>
       <c r="D16" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E16" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="J16" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="K16" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L16" s="2"/>
-    </row>
-    <row r="17" spans="3:12" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M16" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="17" spans="3:13" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C17" s="1"/>
       <c r="D17" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E17" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J17" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I17" s="6" t="s">
+      <c r="K17" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="J17" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K17" s="2" t="s">
+      <c r="L17" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="L17" s="6" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="18" spans="3:12" ht="91.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M17" s="6" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="18" spans="3:13" ht="166.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C18" s="1"/>
       <c r="D18" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E18" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I18" s="6" t="s">
+      <c r="J18" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="J18" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="K18" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="19" spans="3:12" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="M18" s="6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="19" spans="3:13" ht="91.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C19" s="1"/>
       <c r="D19" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E19" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>48</v>
+      <c r="J19" s="6" t="s">
+        <v>47</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="20" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>133</v>
+      </c>
+      <c r="M19" s="6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="20" spans="3:13" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C20" s="1"/>
       <c r="D20" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E20" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H20" s="2" t="s">
+      <c r="I20" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="I20" s="6" t="s">
+      <c r="J20" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="J20" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="K20" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="21" spans="3:12" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+      <c r="M20" s="6" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="21" spans="3:13" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C21" s="1"/>
       <c r="D21" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="K21" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="E21" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="G21" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="I21" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="K21" s="8" t="s">
-        <v>114</v>
-      </c>
       <c r="L21" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="22" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="22" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C22" s="1"/>
       <c r="D22" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F22" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H22" s="2" t="s">
+      <c r="I22" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="I22" s="6" t="s">
+      <c r="J22" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J22" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="K22" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L22" s="2"/>
-    </row>
-    <row r="23" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M22" s="2"/>
+    </row>
+    <row r="23" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C23" s="1"/>
       <c r="D23" s="2"/>
       <c r="E23" s="6"/>
@@ -2500,8 +2309,9 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
-    </row>
-    <row r="24" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M23" s="2"/>
+    </row>
+    <row r="24" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C24" s="1"/>
       <c r="D24" s="2"/>
       <c r="E24" s="6"/>
@@ -2512,8 +2322,9 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
-    </row>
-    <row r="25" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M24" s="2"/>
+    </row>
+    <row r="25" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C25" s="1"/>
       <c r="D25" s="2"/>
       <c r="E25" s="6"/>
@@ -2524,8 +2335,9 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
-    </row>
-    <row r="26" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M25" s="2"/>
+    </row>
+    <row r="26" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C26" s="1"/>
       <c r="D26" s="2"/>
       <c r="E26" s="6"/>
@@ -2536,8 +2348,9 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
-    </row>
-    <row r="27" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M26" s="2"/>
+    </row>
+    <row r="27" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C27" s="1"/>
       <c r="D27" s="2"/>
       <c r="E27" s="6"/>
@@ -2548,8 +2361,9 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
-    </row>
-    <row r="28" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M27" s="2"/>
+    </row>
+    <row r="28" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C28" s="1"/>
       <c r="D28" s="2"/>
       <c r="E28" s="6"/>
@@ -2560,8 +2374,9 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
-    </row>
-    <row r="29" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M28" s="2"/>
+    </row>
+    <row r="29" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C29" s="1"/>
       <c r="D29" s="2"/>
       <c r="E29" s="6"/>
@@ -2572,8 +2387,9 @@
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
-    </row>
-    <row r="30" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M29" s="2"/>
+    </row>
+    <row r="30" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C30" s="1"/>
       <c r="D30" s="2"/>
       <c r="E30" s="6"/>
@@ -2584,8 +2400,9 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
-    </row>
-    <row r="31" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M30" s="2"/>
+    </row>
+    <row r="31" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C31" s="1"/>
       <c r="D31" s="2"/>
       <c r="E31" s="6"/>
@@ -2596,8 +2413,9 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
-    </row>
-    <row r="32" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M31" s="2"/>
+    </row>
+    <row r="32" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C32" s="1"/>
       <c r="D32" s="2"/>
       <c r="E32" s="6"/>
@@ -2608,8 +2426,9 @@
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
-    </row>
-    <row r="33" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M32" s="2"/>
+    </row>
+    <row r="33" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C33" s="1"/>
       <c r="D33" s="2"/>
       <c r="E33" s="6"/>
@@ -2620,8 +2439,9 @@
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
-    </row>
-    <row r="34" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M33" s="2"/>
+    </row>
+    <row r="34" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C34" s="1"/>
       <c r="D34" s="2"/>
       <c r="E34" s="6"/>
@@ -2632,8 +2452,9 @@
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
-    </row>
-    <row r="35" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M34" s="2"/>
+    </row>
+    <row r="35" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C35" s="1"/>
       <c r="D35" s="2"/>
       <c r="E35" s="6"/>
@@ -2644,8 +2465,9 @@
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
-    </row>
-    <row r="36" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M35" s="2"/>
+    </row>
+    <row r="36" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C36" s="1"/>
       <c r="D36" s="2"/>
       <c r="E36" s="6"/>
@@ -2656,8 +2478,9 @@
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
-    </row>
-    <row r="37" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M36" s="2"/>
+    </row>
+    <row r="37" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C37" s="1"/>
       <c r="D37" s="2"/>
       <c r="E37" s="6"/>
@@ -2668,8 +2491,9 @@
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
-    </row>
-    <row r="38" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M37" s="2"/>
+    </row>
+    <row r="38" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C38" s="1"/>
       <c r="D38" s="2"/>
       <c r="E38" s="6"/>
@@ -2680,8 +2504,9 @@
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
-    </row>
-    <row r="39" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M38" s="2"/>
+    </row>
+    <row r="39" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C39" s="1"/>
       <c r="D39" s="2"/>
       <c r="E39" s="6"/>
@@ -2692,8 +2517,9 @@
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
-    </row>
-    <row r="40" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M39" s="2"/>
+    </row>
+    <row r="40" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C40" s="1"/>
       <c r="D40" s="2"/>
       <c r="E40" s="6"/>
@@ -2704,868 +2530,940 @@
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
       <c r="L40" s="8"/>
-    </row>
-    <row r="41" spans="3:12" ht="76.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M40" s="2"/>
+    </row>
+    <row r="41" spans="3:13" ht="76.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C41" s="1"/>
       <c r="D41" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="E41" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="E41" s="9" t="s">
+      <c r="F41" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="F41" s="8" t="s">
+      <c r="G41" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H41" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="G41" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H41" s="8" t="s">
+      <c r="I41" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="I41" s="9" t="s">
+      <c r="J41" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="J41" s="8" t="s">
+      <c r="K41" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="K41" s="8" t="s">
-        <v>143</v>
-      </c>
       <c r="L41" s="8"/>
-    </row>
-    <row r="42" spans="3:12" ht="31.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M41" s="2"/>
+    </row>
+    <row r="42" spans="3:13" ht="31.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C42" s="1"/>
       <c r="D42" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E42" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H42" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="F42" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H42" s="2" t="s">
+      <c r="I42" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="I42" s="6" t="s">
-        <v>146</v>
-      </c>
       <c r="J42" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
-    </row>
-    <row r="43" spans="3:12" ht="46.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M42" s="2"/>
+    </row>
+    <row r="43" spans="3:13" ht="46.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C43" s="1"/>
       <c r="D43" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E43" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I43" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="F43" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I43" s="6" t="s">
+      <c r="J43" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="J43" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="K43" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L43" s="2"/>
-    </row>
-    <row r="44" spans="3:12" ht="31.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M43" s="2"/>
+    </row>
+    <row r="44" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C44" s="1"/>
       <c r="D44" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E44" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I44" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="F44" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I44" s="6" t="s">
+      <c r="J44" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="J44" s="2" t="s">
-        <v>154</v>
-      </c>
       <c r="K44" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L44" s="2"/>
-    </row>
-    <row r="45" spans="3:12" ht="31.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M44" s="2"/>
+    </row>
+    <row r="45" spans="3:13" ht="31.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C45" s="1"/>
       <c r="D45" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E45" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I45" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="F45" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H45" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I45" s="6" t="s">
-        <v>157</v>
-      </c>
       <c r="J45" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L45" s="2"/>
-    </row>
-    <row r="46" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M45" s="2"/>
+    </row>
+    <row r="46" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C46" s="1"/>
       <c r="D46" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E46" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H46" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="F46" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H46" s="2" t="s">
+      <c r="I46" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="I46" s="6" t="s">
-        <v>161</v>
-      </c>
       <c r="J46" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L46" s="2"/>
-    </row>
-    <row r="47" spans="3:12" ht="31.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M46" s="2"/>
+    </row>
+    <row r="47" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C47" s="1"/>
       <c r="D47" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E47" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I47" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="F47" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H47" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I47" s="6" t="s">
+      <c r="J47" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="J47" s="2" t="s">
-        <v>165</v>
-      </c>
       <c r="K47" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L47" s="2"/>
-    </row>
-    <row r="48" spans="3:12" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M47" s="2"/>
+    </row>
+    <row r="48" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C48" s="1"/>
       <c r="D48" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E48" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I48" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="F48" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H48" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I48" s="6" t="s">
-        <v>168</v>
-      </c>
       <c r="J48" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L48" s="2"/>
-    </row>
-    <row r="49" spans="3:12" ht="31.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M48" s="2"/>
+    </row>
+    <row r="49" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C49" s="1"/>
       <c r="D49" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E49" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I49" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F49" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H49" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I49" s="6" t="s">
+      <c r="J49" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="J49" s="2" t="s">
-        <v>172</v>
-      </c>
       <c r="K49" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L49" s="2"/>
-    </row>
-    <row r="50" spans="3:12" ht="31.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M49" s="2"/>
+    </row>
+    <row r="50" spans="3:13" ht="16.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C50" s="1"/>
       <c r="D50" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E50" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I50" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="F50" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H50" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I50" s="6" t="s">
-        <v>175</v>
-      </c>
       <c r="J50" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L50" s="2"/>
-    </row>
-    <row r="51" spans="3:12" ht="31.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M50" s="2"/>
+    </row>
+    <row r="51" spans="3:13" ht="31.5" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C51" s="1"/>
       <c r="D51" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E51" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I51" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="F51" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G51" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H51" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I51" s="6" t="s">
+      <c r="J51" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="J51" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="K51" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L51" s="2"/>
-    </row>
-    <row r="52" spans="3:12" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M51" s="2"/>
+    </row>
+    <row r="52" spans="3:13" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C52" s="1"/>
       <c r="D52" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E52" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="E52" s="6" t="s">
+      <c r="F52" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="F52" s="2" t="s">
+      <c r="G52" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H52" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="G52" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H52" s="2" t="s">
+      <c r="I52" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="I52" s="6" t="s">
+      <c r="J52" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="J52" s="2" t="s">
+      <c r="K52" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="K52" s="2" t="s">
-        <v>143</v>
-      </c>
       <c r="L52" s="2"/>
-    </row>
-    <row r="53" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M52" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="53" spans="3:13" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C53" s="1"/>
       <c r="D53" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E53" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H53" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="F53" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H53" s="2" t="s">
+      <c r="I53" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="I53" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="J53" s="2" t="s">
-        <v>143</v>
+      <c r="J53" s="6" t="s">
+        <v>142</v>
       </c>
       <c r="K53" s="2"/>
       <c r="L53" s="2"/>
-    </row>
-    <row r="54" spans="3:12" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M53" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="54" spans="3:13" ht="61.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C54" s="1"/>
       <c r="D54" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E54" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I54" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="F54" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I54" s="6" t="s">
+      <c r="J54" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="J54" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="K54" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L54" s="2"/>
-    </row>
-    <row r="55" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M54" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="55" spans="3:13" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C55" s="1"/>
       <c r="D55" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E55" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I55" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="F55" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H55" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I55" s="6" t="s">
+      <c r="J55" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="J55" s="2" t="s">
-        <v>154</v>
-      </c>
       <c r="K55" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L55" s="2"/>
-    </row>
-    <row r="56" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M55" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="56" spans="3:13" ht="61.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C56" s="1"/>
       <c r="D56" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E56" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I56" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="F56" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H56" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I56" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="J56" s="2" t="s">
-        <v>35</v>
+      <c r="J56" s="6" t="s">
+        <v>34</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L56" s="2"/>
-    </row>
-    <row r="57" spans="3:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M56" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="57" spans="3:13" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C57" s="1"/>
       <c r="D57" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E57" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H57" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F57" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G57" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H57" s="2" t="s">
+      <c r="I57" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="I57" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="J57" s="2" t="s">
-        <v>154</v>
+      <c r="J57" s="6" t="s">
+        <v>153</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L57" s="2"/>
-    </row>
-    <row r="58" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M57" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="58" spans="3:13" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C58" s="1"/>
       <c r="D58" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E58" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H58" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I58" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="F58" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G58" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H58" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I58" s="6" t="s">
+      <c r="J58" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="J58" s="2" t="s">
-        <v>165</v>
-      </c>
       <c r="K58" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L58" s="2"/>
-    </row>
-    <row r="59" spans="3:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M58" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="59" spans="3:13" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C59" s="1"/>
       <c r="D59" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E59" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I59" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="F59" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G59" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H59" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I59" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="J59" s="2" t="s">
-        <v>154</v>
+      <c r="J59" s="6" t="s">
+        <v>153</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L59" s="2"/>
-    </row>
-    <row r="60" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M59" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="60" spans="3:13" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C60" s="1"/>
       <c r="D60" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E60" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I60" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F60" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H60" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I60" s="6" t="s">
+      <c r="J60" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="J60" s="2" t="s">
-        <v>172</v>
-      </c>
       <c r="K60" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L60" s="2"/>
-    </row>
-    <row r="61" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M60" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="61" spans="3:13" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C61" s="1"/>
       <c r="D61" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E61" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H61" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I61" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="F61" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G61" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H61" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I61" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="J61" s="2" t="s">
-        <v>154</v>
+      <c r="J61" s="6" t="s">
+        <v>153</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L61" s="2"/>
-    </row>
-    <row r="62" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M61" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="62" spans="3:13" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C62" s="1"/>
       <c r="D62" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E62" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H62" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I62" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="F62" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G62" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H62" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I62" s="6" t="s">
+      <c r="J62" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="J62" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="K62" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L62" s="2"/>
-    </row>
-    <row r="63" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M62" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="63" spans="3:13" ht="61.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C63" s="1"/>
       <c r="D63" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E63" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="F63" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G63" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H63" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="F63" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="G63" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H63" s="8" t="s">
+      <c r="I63" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="I63" s="9" t="s">
+      <c r="J63" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="J63" s="8" t="s">
-        <v>184</v>
-      </c>
       <c r="K63" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L63" s="8"/>
-    </row>
-    <row r="64" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M63" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="64" spans="3:13" ht="61.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C64" s="1"/>
       <c r="D64" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E64" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="F64" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="F64" s="2" t="s">
+      <c r="G64" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H64" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="G64" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H64" s="2" t="s">
+      <c r="I64" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="I64" s="6" t="s">
+      <c r="J64" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="J64" s="2" t="s">
-        <v>190</v>
-      </c>
       <c r="K64" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L64" s="2"/>
-    </row>
-    <row r="65" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M64" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="65" spans="3:13" ht="61.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C65" s="1"/>
       <c r="D65" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E65" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H65" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="F65" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="G65" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H65" s="2" t="s">
+      <c r="I65" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="I65" s="6" t="s">
+      <c r="J65" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="J65" s="2" t="s">
-        <v>195</v>
-      </c>
       <c r="K65" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L65" s="2"/>
-    </row>
-    <row r="66" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M65" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="66" spans="3:13" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C66" s="1"/>
       <c r="D66" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E66" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F66" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H66" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H66" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="I66" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="I66" s="8" t="s">
+      <c r="J66" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="J66" s="9" t="s">
-        <v>201</v>
-      </c>
       <c r="K66" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L66" s="8"/>
-    </row>
-    <row r="67" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M66" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="67" spans="3:13" ht="91.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C67" s="1"/>
       <c r="D67" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E67" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="E67" s="6" t="s">
+      <c r="F67" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="F67" s="2" t="s">
+      <c r="G67" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="G67" s="2" t="s">
+      <c r="H67" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="H67" s="2" t="s">
+      <c r="I67" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="I67" s="6" t="s">
+      <c r="J67" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="J67" s="2" t="s">
-        <v>208</v>
-      </c>
       <c r="K67" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L67" s="2"/>
-    </row>
-    <row r="68" spans="3:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M67" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="68" spans="3:13" ht="61.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C68" s="1"/>
       <c r="D68" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E68" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="E68" s="6" t="s">
+      <c r="F68" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="F68" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="G68" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H68" s="2" t="s">
+      <c r="I68" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="I68" s="6" t="s">
+      <c r="J68" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="J68" s="2" t="s">
-        <v>213</v>
-      </c>
       <c r="K68" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L68" s="2"/>
-    </row>
-    <row r="69" spans="3:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M68" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="69" spans="3:13" ht="61.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C69" s="1"/>
       <c r="D69" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E69" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="E69" s="6" t="s">
+      <c r="F69" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H69" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="F69" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="G69" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H69" s="2" t="s">
+      <c r="I69" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="I69" s="6" t="s">
+      <c r="J69" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="J69" s="2" t="s">
-        <v>218</v>
-      </c>
       <c r="K69" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L69" s="2"/>
-    </row>
-    <row r="70" spans="3:12" ht="61.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M69" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="70" spans="3:13" ht="91.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C70" s="1"/>
       <c r="D70" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="E70" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="E70" s="9" t="s">
+      <c r="F70" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="G70" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="H70" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="F70" s="8" t="s">
-        <v>204</v>
-      </c>
-      <c r="G70" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="H70" s="8" t="s">
+      <c r="I70" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="I70" s="9" t="s">
+      <c r="J70" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="J70" s="8" t="s">
-        <v>223</v>
-      </c>
       <c r="K70" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="L70" s="8"/>
-    </row>
-    <row r="71" spans="3:12" ht="30.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="M70" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="71" spans="3:13" ht="60.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C71" s="1"/>
       <c r="D71" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="E71" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="F71" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="E71" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="F71" s="8" t="s">
+      <c r="G71" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H71" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="G71" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H71" s="8" t="s">
+      <c r="I71" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="I71" s="9" t="s">
+      <c r="J71" s="9" t="s">
         <v>227</v>
-      </c>
-      <c r="J71" s="8" t="s">
-        <v>228</v>
       </c>
       <c r="K71" s="8"/>
       <c r="L71" s="8"/>
+      <c r="M71" s="8" t="s">
+        <v>231</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="K5:K21">
@@ -3597,8 +3495,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3616,17 +3515,17 @@
   <sheetData>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -3637,35 +3536,35 @@
         <v>0</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C8" s="10">
         <v>40</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>71</v>
-      </c>
       <c r="C9" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
@@ -3673,7 +3572,7 @@
     <row r="11" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
@@ -3684,35 +3583,35 @@
         <v>0</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C13" s="10">
         <v>120</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>71</v>
-      </c>
       <c r="C14" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
@@ -3720,7 +3619,7 @@
     <row r="16" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="17" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B17" s="13"/>
     </row>
@@ -3729,21 +3628,21 @@
         <v>0</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B19" s="10" t="s">
         <v>70</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B21" s="13"/>
     </row>
@@ -3752,29 +3651,29 @@
         <v>0</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -3782,38 +3681,38 @@
     </row>
     <row r="27" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B27" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B27" s="10" t="s">
-        <v>82</v>
-      </c>
       <c r="C27" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" s="10" t="s">
         <v>79</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B28" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="B28" s="10" t="s">
-        <v>71</v>
-      </c>
       <c r="C28" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B29" s="14" t="s">
         <v>91</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>92</v>
       </c>
       <c r="C29" s="14"/>
       <c r="D29" s="14"/>
@@ -3821,17 +3720,17 @@
     <row r="30" spans="1:4" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B33" s="11">
         <v>2958465.999988426</v>
@@ -3839,16 +3738,16 @@
     </row>
     <row r="35" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="13" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B35" s="13"/>
     </row>
     <row r="36" spans="1:2" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B36" s="10" t="s">
         <v>84</v>
-      </c>
-      <c r="B36" s="10" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -3865,417 +3764,4 @@
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C4DA4C7-33A9-464F-992B-3F3EED701EC5}">
-  <dimension ref="B2:K16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="2.28515625" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" customWidth="1"/>
-    <col min="4" max="4" width="29.140625" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="88.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="33.7109375" customWidth="1"/>
-    <col min="9" max="9" width="20.140625" customWidth="1"/>
-    <col min="10" max="10" width="23.85546875" customWidth="1"/>
-    <col min="11" max="11" width="29.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:11" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-    </row>
-    <row r="3" spans="2:11" ht="36" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="3"/>
-      <c r="C3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="2:11" ht="76.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="1"/>
-      <c r="C4" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="K4" s="8"/>
-    </row>
-    <row r="5" spans="2:11" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="1"/>
-      <c r="C5" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-    </row>
-    <row r="6" spans="2:11" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="1"/>
-      <c r="C6" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="K6" s="2"/>
-    </row>
-    <row r="7" spans="2:11" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="1"/>
-      <c r="C7" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="K7" s="2"/>
-    </row>
-    <row r="8" spans="2:11" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="1"/>
-      <c r="C8" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="K8" s="2"/>
-    </row>
-    <row r="9" spans="2:11" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="1"/>
-      <c r="C9" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="K9" s="2"/>
-    </row>
-    <row r="10" spans="2:11" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="1"/>
-      <c r="C10" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="K10" s="2"/>
-    </row>
-    <row r="11" spans="2:11" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="1"/>
-      <c r="C11" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="K11" s="2"/>
-    </row>
-    <row r="12" spans="2:11" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="1"/>
-      <c r="C12" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="K12" s="2"/>
-    </row>
-    <row r="13" spans="2:11" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="1"/>
-      <c r="C13" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="K13" s="2"/>
-    </row>
-    <row r="14" spans="2:11" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="1"/>
-      <c r="C14" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="K14" s="2"/>
-    </row>
-    <row r="15" spans="2:11" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="1"/>
-      <c r="C15" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="K15" s="2"/>
-    </row>
-    <row r="16" spans="2:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-  </sheetData>
-  <conditionalFormatting sqref="J4:J15">
-    <cfRule type="expression" dxfId="0" priority="4">
-      <formula>$K4="Not started"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F15" xr:uid="{640253AE-59FE-4D3F-AE26-80BE02D1BC65}">
-      <formula1>"P.E, V.L, T.D"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>